<commit_message>
feat: Add Auto-Magic Logger, inline category, splash screen
</commit_message>
<xml_diff>
--- a/test/Expense Tracker Testing Sheet.xlsx
+++ b/test/Expense Tracker Testing Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Amey\Projects\Flutter Projects\Expense_Tracker\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC66083-1111-433A-865C-86A6D4FE7C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED9ABAC5-C524-4014-9F7A-5A8A0E08B0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D2AA2B50-82DF-4489-9982-C8493A994DFB}"/>
   </bookViews>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="111">
   <si>
     <t>Names of users</t>
   </si>
@@ -149,38 +171,235 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Bug</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Subcribtion Cant be edited after adding them, they can only be deleted</t>
-  </si>
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>She says she can make 2 same entries for Subscription</t>
-  </si>
-  <si>
-    <t>Module</t>
+    <t>Email Address</t>
+  </si>
+  <si>
+    <t>Downloaded</t>
+  </si>
+  <si>
+    <t>Screen / Module</t>
+  </si>
+  <si>
+    <t>Sugestions</t>
+  </si>
+  <si>
+    <t>Bugs</t>
+  </si>
+  <si>
+    <t>Amey Bhogle</t>
+  </si>
+  <si>
+    <t>amey.bhogle12@gmail.com</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Nimish Malekar</t>
+  </si>
+  <si>
+    <t>nimishmalekar28258@gmail.com</t>
+  </si>
+  <si>
+    <t>Link Sent</t>
+  </si>
+  <si>
+    <t>suhoney03@gmail.com</t>
+  </si>
+  <si>
+    <t>Sharvil</t>
+  </si>
+  <si>
+    <t>sharvil.palvekar@gmail.com</t>
+  </si>
+  <si>
+    <t>Add a UPI Payment option in this app itself.</t>
+  </si>
+  <si>
+    <t>anthony242002@gmail.com</t>
+  </si>
+  <si>
+    <t>Hemant Sharma</t>
+  </si>
+  <si>
+    <t>hemantborn82@gmail.com</t>
+  </si>
+  <si>
+    <t>Desmond</t>
+  </si>
+  <si>
+    <t>ferraodesmond122asis@gmail.com</t>
+  </si>
+  <si>
+    <t>Soham Morlikar</t>
+  </si>
+  <si>
+    <t>sohamorlikar@gmail.com</t>
+  </si>
+  <si>
+    <t>Mummy</t>
+  </si>
+  <si>
+    <t>neha.bhogle36@gmail.com</t>
+  </si>
+  <si>
+    <t>Ishika</t>
+  </si>
+  <si>
+    <t>ishika.bhogle2008@gmail.com</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>ameyvshinde@gmail.com</t>
+  </si>
+  <si>
+    <t>Pappa</t>
+  </si>
+  <si>
+    <t>amey.lic123@gmail.com</t>
+  </si>
+  <si>
+    <t>Vedant Sawant</t>
+  </si>
+  <si>
+    <t>vs9833211034@gmail.com</t>
+  </si>
+  <si>
+    <t>Manjyot Jogle</t>
+  </si>
+  <si>
+    <t>lucywilson08@gmail.com</t>
+  </si>
+  <si>
+    <t>Pooja</t>
+  </si>
+  <si>
+    <t>poojaagre210@gmail.com</t>
+  </si>
+  <si>
+    <t>Shriraj</t>
+  </si>
+  <si>
+    <t>shriraj1223shetty@gmail.com</t>
+  </si>
+  <si>
+    <t>ishitashetty127@gmail.com</t>
+  </si>
+  <si>
+    <t>guptakhushboo2153@gmail.com</t>
+  </si>
+  <si>
+    <t>Prathamesh Surve</t>
+  </si>
+  <si>
+    <t>prathameshhsurvee928@gmail.com</t>
+  </si>
+  <si>
+    <t>Sahil Sayyed</t>
+  </si>
+  <si>
+    <t>sahilsayyed0409@gmail.com</t>
+  </si>
+  <si>
+    <t>Yogesh (Nemo Friend)</t>
+  </si>
+  <si>
+    <t>patwalyogesh7@gmail.com</t>
+  </si>
+  <si>
+    <t>Bhakti</t>
+  </si>
+  <si>
+    <t>bhaktiwaghamare@gmail.com</t>
+  </si>
+  <si>
+    <t>Tejal</t>
+  </si>
+  <si>
+    <t>tejalvaprajpersonal@gmail.com</t>
+  </si>
+  <si>
+    <t>Snehal Borji</t>
+  </si>
+  <si>
+    <t>snehalborji933@gmail.com</t>
+  </si>
+  <si>
+    <t>Sharon</t>
+  </si>
+  <si>
+    <t>sharonmavelil03@gmail.com</t>
+  </si>
+  <si>
+    <t>Bhavya</t>
+  </si>
+  <si>
+    <t>doshibhavya961@gmail.com</t>
+  </si>
+  <si>
+    <t>Chart Screen</t>
+  </si>
+  <si>
+    <t>Add a calendar icon and a calender to select the date at the very top. It is annoying to keep tapping to go back to check the Data.</t>
+  </si>
+  <si>
+    <t>Home Screen (Add transaction Dialog)</t>
+  </si>
+  <si>
+    <t>There is a "$" symbol beside the income text, if i select INR from the settings the dollar icon should not be here it was supposed to be a "Rupee" symbol.
+(Small detail caught by him, not a big deal but worth looking into)</t>
+  </si>
+  <si>
+    <t>The X-axis onthe line graph shows names of the moths (Jan Feb March etc,) Regardless of what is selected (this month, Last month, last three months, Year to date. It should Vary according to option selected.</t>
+  </si>
+  <si>
+    <t>Over All</t>
+  </si>
+  <si>
+    <t>Settings (Auth)</t>
+  </si>
+  <si>
+    <t>When the authentication is turened on from the settings, and taken a screenshot. The app gets locked everytime you take a screen shot.</t>
+  </si>
+  <si>
+    <t>the walltet slider has 3 wallet cards initially. Similarly it has 3 small dots bellow it indicatinf the card at which we are. The small dots never reach the third dot even thought there are 3 wallets. It gets stopped at 2nd dot.</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Leve (Austrailia)</t>
+  </si>
+  <si>
+    <t>I added 11000 INR then deleted it and changed the currency to AUD. I continued with some transaction after that. But the chart's Line Graph is still showing that 11000 INR entry, it didn’t got reflected when I deleted the INR amount.</t>
+  </si>
+  <si>
+    <t>Split Screen</t>
+  </si>
+  <si>
+    <t>Multi Player Split by sending links</t>
+  </si>
+  <si>
+    <t>Subscription Screen</t>
+  </si>
+  <si>
+    <t>Images of the Suggestions (From other app)</t>
+  </si>
+  <si>
+    <t>Your app shows all the amount together in the donut chart. The app I use shows the amount spent on that categoty when clicked on that category , It’s a suggestion you can add that in your app as well</t>
+  </si>
+  <si>
+    <t>1. If I have canceled a subcription of netflix, there are high changes that I will forgot to remove that from your app. So you can add a notification for the upcoming subscription so that I'll know that ohh I have to cancel uit from this  app
+2. Also it show the number of transaction done with this category, and when clicked on that it should filter that categories transation and show me those categories transaction.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,8 +437,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -228,30 +468,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -261,50 +483,37 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -330,207 +539,109 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="19">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.59999389629810485"/>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.59999389629810485"/>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -729,37 +840,86 @@
 </styleSheet>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65B549F6-FEC8-4836-B547-DAFC95B92456}" name="Table1" displayName="Table1" ref="B3:K24" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65B549F6-FEC8-4836-B547-DAFC95B92456}" name="Table1" displayName="Table1" ref="B3:K24" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="B3:K24" xr:uid="{65B549F6-FEC8-4836-B547-DAFC95B92456}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{515BF0C7-B046-4F1D-8837-F861091D76B4}" name="Sr. no" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{64CC9BE8-E2FA-4B09-94BA-B8C1D6E28097}" name="Names of users" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{F03775AC-0CFF-43B2-B8F3-271830FE0C9B}" name="Platform" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{360B2055-7B5D-4695-AD7E-0E1EBF0156E3}" name="Device" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{0F14A130-C3E9-4CE6-96CD-523B20C7E3F1}" name="APK  sent date" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{4176BADB-9A8D-40BD-AFE8-3EEADA740F23}" name="Testing Status" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{8AAD5452-F805-4F1E-92D7-7218C30CDB85}" name="Last Follow-up Date" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{BD593D3D-A6C6-4E79-AAC3-E92695A02C72}" name="Form Submitted?" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{AB132D5A-BC09-4E06-88C7-344A09A9C1B0}" name="Playstore Email ID" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{32094475-90BF-41DD-9AFF-097673DC4275}" name="Opted-in to Play Store Test?" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{515BF0C7-B046-4F1D-8837-F861091D76B4}" name="Sr. no" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{64CC9BE8-E2FA-4B09-94BA-B8C1D6E28097}" name="Names of users" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{F03775AC-0CFF-43B2-B8F3-271830FE0C9B}" name="Platform" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{360B2055-7B5D-4695-AD7E-0E1EBF0156E3}" name="Device" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{0F14A130-C3E9-4CE6-96CD-523B20C7E3F1}" name="APK  sent date" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{4176BADB-9A8D-40BD-AFE8-3EEADA740F23}" name="Testing Status" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{8AAD5452-F805-4F1E-92D7-7218C30CDB85}" name="Last Follow-up Date" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{BD593D3D-A6C6-4E79-AAC3-E92695A02C72}" name="Form Submitted?" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{AB132D5A-BC09-4E06-88C7-344A09A9C1B0}" name="Playstore Email ID" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{32094475-90BF-41DD-9AFF-097673DC4275}" name="Opted-in to Play Store Test?" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7AFBD477-9A8A-4574-8531-EC2A870BE2A3}" name="Table2" displayName="Table2" ref="B3:G25" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="B3:G25" xr:uid="{7AFBD477-9A8A-4574-8531-EC2A870BE2A3}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{41A0D799-7828-4F60-B2ED-6C7B64C2AB1D}" name="Name" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{34AEA048-73E2-45AE-AB3A-7A480571098B}" name="Module" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{DB19F42C-90F9-48FB-A6D9-21FB0F9B9A94}" name="Type" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{9A801F71-70D5-4AC8-9993-501158102F09}" name="Description" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{11203C2D-EE74-45AD-A6EF-D7495C3D389D}" name="Priority" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{D66F2BEB-021A-4377-8EDA-DE66AF687C4D}" name="Column1" dataDxfId="3"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1572,36 +1732,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA36B7C3-60B0-4756-9A31-26CCACF4EEE1}">
-  <dimension ref="B3:O25"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultRowHeight="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" style="15" customWidth="1"/>
     <col min="5" max="5" width="55.109375" customWidth="1"/>
-    <col min="6" max="6" width="19.5546875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" customWidth="1"/>
+    <col min="6" max="6" width="53.5546875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="29.77734375" style="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
+    <row r="1" spans="1:15" s="26" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="B1" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="21"/>
+    </row>
+    <row r="3" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>42</v>
-      </c>
+      <c r="B3" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="23"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
@@ -1611,15 +1804,20 @@
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
     </row>
-    <row r="4" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="11"/>
+    <row r="4" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="24"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
@@ -1629,15 +1827,24 @@
       <c r="N4" s="8"/>
       <c r="O4" s="8"/>
     </row>
-    <row r="5" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="11"/>
+    <row r="5" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="21"/>
+      <c r="G5" s="24"/>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
@@ -1647,15 +1854,28 @@
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="11"/>
+    <row r="6" spans="1:15" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="G6" s="13" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
@@ -1665,15 +1885,18 @@
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
-    <row r="7" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="11"/>
+    <row r="7" spans="1:15" ht="105.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" s="21"/>
+      <c r="G7" s="24"/>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
@@ -1683,15 +1906,18 @@
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
     </row>
-    <row r="8" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="11"/>
+    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="24"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
@@ -1701,15 +1927,20 @@
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="11"/>
+    <row r="9" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
@@ -1719,15 +1950,20 @@
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
     </row>
-    <row r="10" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="11"/>
+    <row r="10" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="24"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
@@ -1737,15 +1973,18 @@
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
     </row>
-    <row r="11" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="11"/>
+    <row r="11" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="24"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
@@ -1755,15 +1994,20 @@
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
     </row>
-    <row r="12" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="11"/>
+    <row r="12" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
@@ -1773,21 +2017,20 @@
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
     </row>
-    <row r="13" spans="2:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="11"/>
+    <row r="13" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
@@ -1797,17 +2040,20 @@
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
     </row>
-    <row r="14" spans="2:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="18"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="11" t="s">
+    <row r="14" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="9"/>
-      <c r="G14" s="11"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="24"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
@@ -1817,15 +2063,20 @@
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
     </row>
-    <row r="15" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="11"/>
+    <row r="15" spans="1:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="24"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
@@ -1835,15 +2086,20 @@
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
     </row>
-    <row r="16" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="11"/>
+    <row r="16" spans="1:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="24"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
@@ -1853,15 +2109,20 @@
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
     </row>
-    <row r="17" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="11"/>
+    <row r="17" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="24"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
       <c r="J17" s="8"/>
@@ -1871,15 +2132,20 @@
       <c r="N17" s="8"/>
       <c r="O17" s="8"/>
     </row>
-    <row r="18" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="11"/>
+    <row r="18" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="24"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
       <c r="J18" s="8"/>
@@ -1889,15 +2155,20 @@
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
     </row>
-    <row r="19" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="11"/>
+    <row r="19" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="24"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
       <c r="J19" s="8"/>
@@ -1907,13 +2178,20 @@
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
     </row>
-    <row r="20" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="16"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="11"/>
+    <row r="20" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="24"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
       <c r="J20" s="8"/>
@@ -1923,13 +2201,20 @@
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
     </row>
-    <row r="21" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="21"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="11"/>
+    <row r="21" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
@@ -1939,13 +2224,20 @@
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
     </row>
-    <row r="22" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="16"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="11"/>
+    <row r="22" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="24"/>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
@@ -1955,13 +2247,20 @@
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
     </row>
-    <row r="23" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="21"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="11"/>
+    <row r="23" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="24"/>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
       <c r="J23" s="8"/>
@@ -1971,13 +2270,20 @@
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
     </row>
-    <row r="24" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="16"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="11"/>
+    <row r="24" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
@@ -1987,13 +2293,20 @@
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
     </row>
-    <row r="25" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="11"/>
+    <row r="25" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="24"/>
       <c r="H25" s="8"/>
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
@@ -2003,10 +2316,138 @@
       <c r="N25" s="8"/>
       <c r="O25" s="8"/>
     </row>
+    <row r="26" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+    </row>
+    <row r="27" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+    </row>
+    <row r="28" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="21"/>
+    </row>
+    <row r="29" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="16"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$C2="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A82">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$C2="No"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>$C2="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{FFA2BD12-D726-4B56-B8E9-BC6E0D925A91}">
+      <formula1>"Yes, No, Link Sent"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Free version improvements - Splash screen, Charts fix, Add Wallet & Category inline
</commit_message>
<xml_diff>
--- a/test/Expense Tracker Testing Sheet.xlsx
+++ b/test/Expense Tracker Testing Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Amey\Projects\Flutter Projects\Expense_Tracker\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC66083-1111-433A-865C-86A6D4FE7C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED9ABAC5-C524-4014-9F7A-5A8A0E08B0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D2AA2B50-82DF-4489-9982-C8493A994DFB}"/>
   </bookViews>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="111">
   <si>
     <t>Names of users</t>
   </si>
@@ -149,38 +171,235 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Bug</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Subcribtion Cant be edited after adding them, they can only be deleted</t>
-  </si>
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>She says she can make 2 same entries for Subscription</t>
-  </si>
-  <si>
-    <t>Module</t>
+    <t>Email Address</t>
+  </si>
+  <si>
+    <t>Downloaded</t>
+  </si>
+  <si>
+    <t>Screen / Module</t>
+  </si>
+  <si>
+    <t>Sugestions</t>
+  </si>
+  <si>
+    <t>Bugs</t>
+  </si>
+  <si>
+    <t>Amey Bhogle</t>
+  </si>
+  <si>
+    <t>amey.bhogle12@gmail.com</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Nimish Malekar</t>
+  </si>
+  <si>
+    <t>nimishmalekar28258@gmail.com</t>
+  </si>
+  <si>
+    <t>Link Sent</t>
+  </si>
+  <si>
+    <t>suhoney03@gmail.com</t>
+  </si>
+  <si>
+    <t>Sharvil</t>
+  </si>
+  <si>
+    <t>sharvil.palvekar@gmail.com</t>
+  </si>
+  <si>
+    <t>Add a UPI Payment option in this app itself.</t>
+  </si>
+  <si>
+    <t>anthony242002@gmail.com</t>
+  </si>
+  <si>
+    <t>Hemant Sharma</t>
+  </si>
+  <si>
+    <t>hemantborn82@gmail.com</t>
+  </si>
+  <si>
+    <t>Desmond</t>
+  </si>
+  <si>
+    <t>ferraodesmond122asis@gmail.com</t>
+  </si>
+  <si>
+    <t>Soham Morlikar</t>
+  </si>
+  <si>
+    <t>sohamorlikar@gmail.com</t>
+  </si>
+  <si>
+    <t>Mummy</t>
+  </si>
+  <si>
+    <t>neha.bhogle36@gmail.com</t>
+  </si>
+  <si>
+    <t>Ishika</t>
+  </si>
+  <si>
+    <t>ishika.bhogle2008@gmail.com</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>ameyvshinde@gmail.com</t>
+  </si>
+  <si>
+    <t>Pappa</t>
+  </si>
+  <si>
+    <t>amey.lic123@gmail.com</t>
+  </si>
+  <si>
+    <t>Vedant Sawant</t>
+  </si>
+  <si>
+    <t>vs9833211034@gmail.com</t>
+  </si>
+  <si>
+    <t>Manjyot Jogle</t>
+  </si>
+  <si>
+    <t>lucywilson08@gmail.com</t>
+  </si>
+  <si>
+    <t>Pooja</t>
+  </si>
+  <si>
+    <t>poojaagre210@gmail.com</t>
+  </si>
+  <si>
+    <t>Shriraj</t>
+  </si>
+  <si>
+    <t>shriraj1223shetty@gmail.com</t>
+  </si>
+  <si>
+    <t>ishitashetty127@gmail.com</t>
+  </si>
+  <si>
+    <t>guptakhushboo2153@gmail.com</t>
+  </si>
+  <si>
+    <t>Prathamesh Surve</t>
+  </si>
+  <si>
+    <t>prathameshhsurvee928@gmail.com</t>
+  </si>
+  <si>
+    <t>Sahil Sayyed</t>
+  </si>
+  <si>
+    <t>sahilsayyed0409@gmail.com</t>
+  </si>
+  <si>
+    <t>Yogesh (Nemo Friend)</t>
+  </si>
+  <si>
+    <t>patwalyogesh7@gmail.com</t>
+  </si>
+  <si>
+    <t>Bhakti</t>
+  </si>
+  <si>
+    <t>bhaktiwaghamare@gmail.com</t>
+  </si>
+  <si>
+    <t>Tejal</t>
+  </si>
+  <si>
+    <t>tejalvaprajpersonal@gmail.com</t>
+  </si>
+  <si>
+    <t>Snehal Borji</t>
+  </si>
+  <si>
+    <t>snehalborji933@gmail.com</t>
+  </si>
+  <si>
+    <t>Sharon</t>
+  </si>
+  <si>
+    <t>sharonmavelil03@gmail.com</t>
+  </si>
+  <si>
+    <t>Bhavya</t>
+  </si>
+  <si>
+    <t>doshibhavya961@gmail.com</t>
+  </si>
+  <si>
+    <t>Chart Screen</t>
+  </si>
+  <si>
+    <t>Add a calendar icon and a calender to select the date at the very top. It is annoying to keep tapping to go back to check the Data.</t>
+  </si>
+  <si>
+    <t>Home Screen (Add transaction Dialog)</t>
+  </si>
+  <si>
+    <t>There is a "$" symbol beside the income text, if i select INR from the settings the dollar icon should not be here it was supposed to be a "Rupee" symbol.
+(Small detail caught by him, not a big deal but worth looking into)</t>
+  </si>
+  <si>
+    <t>The X-axis onthe line graph shows names of the moths (Jan Feb March etc,) Regardless of what is selected (this month, Last month, last three months, Year to date. It should Vary according to option selected.</t>
+  </si>
+  <si>
+    <t>Over All</t>
+  </si>
+  <si>
+    <t>Settings (Auth)</t>
+  </si>
+  <si>
+    <t>When the authentication is turened on from the settings, and taken a screenshot. The app gets locked everytime you take a screen shot.</t>
+  </si>
+  <si>
+    <t>the walltet slider has 3 wallet cards initially. Similarly it has 3 small dots bellow it indicatinf the card at which we are. The small dots never reach the third dot even thought there are 3 wallets. It gets stopped at 2nd dot.</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Leve (Austrailia)</t>
+  </si>
+  <si>
+    <t>I added 11000 INR then deleted it and changed the currency to AUD. I continued with some transaction after that. But the chart's Line Graph is still showing that 11000 INR entry, it didn’t got reflected when I deleted the INR amount.</t>
+  </si>
+  <si>
+    <t>Split Screen</t>
+  </si>
+  <si>
+    <t>Multi Player Split by sending links</t>
+  </si>
+  <si>
+    <t>Subscription Screen</t>
+  </si>
+  <si>
+    <t>Images of the Suggestions (From other app)</t>
+  </si>
+  <si>
+    <t>Your app shows all the amount together in the donut chart. The app I use shows the amount spent on that categoty when clicked on that category , It’s a suggestion you can add that in your app as well</t>
+  </si>
+  <si>
+    <t>1. If I have canceled a subcription of netflix, there are high changes that I will forgot to remove that from your app. So you can add a notification for the upcoming subscription so that I'll know that ohh I have to cancel uit from this  app
+2. Also it show the number of transaction done with this category, and when clicked on that it should filter that categories transation and show me those categories transaction.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,8 +437,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -228,30 +468,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -261,50 +483,37 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -330,207 +539,109 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="19">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.59999389629810485"/>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.59999389629810485"/>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -729,37 +840,86 @@
 </styleSheet>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65B549F6-FEC8-4836-B547-DAFC95B92456}" name="Table1" displayName="Table1" ref="B3:K24" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65B549F6-FEC8-4836-B547-DAFC95B92456}" name="Table1" displayName="Table1" ref="B3:K24" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="B3:K24" xr:uid="{65B549F6-FEC8-4836-B547-DAFC95B92456}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{515BF0C7-B046-4F1D-8837-F861091D76B4}" name="Sr. no" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{64CC9BE8-E2FA-4B09-94BA-B8C1D6E28097}" name="Names of users" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{F03775AC-0CFF-43B2-B8F3-271830FE0C9B}" name="Platform" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{360B2055-7B5D-4695-AD7E-0E1EBF0156E3}" name="Device" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{0F14A130-C3E9-4CE6-96CD-523B20C7E3F1}" name="APK  sent date" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{4176BADB-9A8D-40BD-AFE8-3EEADA740F23}" name="Testing Status" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{8AAD5452-F805-4F1E-92D7-7218C30CDB85}" name="Last Follow-up Date" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{BD593D3D-A6C6-4E79-AAC3-E92695A02C72}" name="Form Submitted?" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{AB132D5A-BC09-4E06-88C7-344A09A9C1B0}" name="Playstore Email ID" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{32094475-90BF-41DD-9AFF-097673DC4275}" name="Opted-in to Play Store Test?" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{515BF0C7-B046-4F1D-8837-F861091D76B4}" name="Sr. no" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{64CC9BE8-E2FA-4B09-94BA-B8C1D6E28097}" name="Names of users" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{F03775AC-0CFF-43B2-B8F3-271830FE0C9B}" name="Platform" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{360B2055-7B5D-4695-AD7E-0E1EBF0156E3}" name="Device" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{0F14A130-C3E9-4CE6-96CD-523B20C7E3F1}" name="APK  sent date" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{4176BADB-9A8D-40BD-AFE8-3EEADA740F23}" name="Testing Status" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{8AAD5452-F805-4F1E-92D7-7218C30CDB85}" name="Last Follow-up Date" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{BD593D3D-A6C6-4E79-AAC3-E92695A02C72}" name="Form Submitted?" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{AB132D5A-BC09-4E06-88C7-344A09A9C1B0}" name="Playstore Email ID" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{32094475-90BF-41DD-9AFF-097673DC4275}" name="Opted-in to Play Store Test?" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7AFBD477-9A8A-4574-8531-EC2A870BE2A3}" name="Table2" displayName="Table2" ref="B3:G25" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="B3:G25" xr:uid="{7AFBD477-9A8A-4574-8531-EC2A870BE2A3}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{41A0D799-7828-4F60-B2ED-6C7B64C2AB1D}" name="Name" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{34AEA048-73E2-45AE-AB3A-7A480571098B}" name="Module" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{DB19F42C-90F9-48FB-A6D9-21FB0F9B9A94}" name="Type" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{9A801F71-70D5-4AC8-9993-501158102F09}" name="Description" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{11203C2D-EE74-45AD-A6EF-D7495C3D389D}" name="Priority" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{D66F2BEB-021A-4377-8EDA-DE66AF687C4D}" name="Column1" dataDxfId="3"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1572,36 +1732,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA36B7C3-60B0-4756-9A31-26CCACF4EEE1}">
-  <dimension ref="B3:O25"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultRowHeight="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" style="15" customWidth="1"/>
     <col min="5" max="5" width="55.109375" customWidth="1"/>
-    <col min="6" max="6" width="19.5546875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" customWidth="1"/>
+    <col min="6" max="6" width="53.5546875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="29.77734375" style="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
+    <row r="1" spans="1:15" s="26" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="B1" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="21"/>
+    </row>
+    <row r="3" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>42</v>
-      </c>
+      <c r="B3" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="23"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
@@ -1611,15 +1804,20 @@
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
     </row>
-    <row r="4" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="11"/>
+    <row r="4" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="24"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
@@ -1629,15 +1827,24 @@
       <c r="N4" s="8"/>
       <c r="O4" s="8"/>
     </row>
-    <row r="5" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="11"/>
+    <row r="5" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="21"/>
+      <c r="G5" s="24"/>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
@@ -1647,15 +1854,28 @@
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="11"/>
+    <row r="6" spans="1:15" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="G6" s="13" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
@@ -1665,15 +1885,18 @@
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
-    <row r="7" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="11"/>
+    <row r="7" spans="1:15" ht="105.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" s="21"/>
+      <c r="G7" s="24"/>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
@@ -1683,15 +1906,18 @@
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
     </row>
-    <row r="8" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="11"/>
+    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="24"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
@@ -1701,15 +1927,20 @@
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="11"/>
+    <row r="9" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
@@ -1719,15 +1950,20 @@
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
     </row>
-    <row r="10" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="11"/>
+    <row r="10" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="24"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
@@ -1737,15 +1973,18 @@
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
     </row>
-    <row r="11" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="11"/>
+    <row r="11" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="24"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
@@ -1755,15 +1994,20 @@
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
     </row>
-    <row r="12" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="11"/>
+    <row r="12" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
@@ -1773,21 +2017,20 @@
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
     </row>
-    <row r="13" spans="2:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="11"/>
+    <row r="13" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
@@ -1797,17 +2040,20 @@
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
     </row>
-    <row r="14" spans="2:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="18"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="11" t="s">
+    <row r="14" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="9"/>
-      <c r="G14" s="11"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="24"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
@@ -1817,15 +2063,20 @@
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
     </row>
-    <row r="15" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="11"/>
+    <row r="15" spans="1:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="24"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
@@ -1835,15 +2086,20 @@
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
     </row>
-    <row r="16" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="11"/>
+    <row r="16" spans="1:15" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="24"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
@@ -1853,15 +2109,20 @@
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
     </row>
-    <row r="17" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="11"/>
+    <row r="17" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="24"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
       <c r="J17" s="8"/>
@@ -1871,15 +2132,20 @@
       <c r="N17" s="8"/>
       <c r="O17" s="8"/>
     </row>
-    <row r="18" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="11"/>
+    <row r="18" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="24"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
       <c r="J18" s="8"/>
@@ -1889,15 +2155,20 @@
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
     </row>
-    <row r="19" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="11"/>
+    <row r="19" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="24"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
       <c r="J19" s="8"/>
@@ -1907,13 +2178,20 @@
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
     </row>
-    <row r="20" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="16"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="11"/>
+    <row r="20" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="24"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
       <c r="J20" s="8"/>
@@ -1923,13 +2201,20 @@
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
     </row>
-    <row r="21" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="21"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="11"/>
+    <row r="21" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
@@ -1939,13 +2224,20 @@
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
     </row>
-    <row r="22" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="16"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="11"/>
+    <row r="22" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="24"/>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
@@ -1955,13 +2247,20 @@
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
     </row>
-    <row r="23" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="21"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="11"/>
+    <row r="23" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="24"/>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
       <c r="J23" s="8"/>
@@ -1971,13 +2270,20 @@
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
     </row>
-    <row r="24" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="16"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="11"/>
+    <row r="24" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
@@ -1987,13 +2293,20 @@
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
     </row>
-    <row r="25" spans="2:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="11"/>
+    <row r="25" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="24"/>
       <c r="H25" s="8"/>
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
@@ -2003,10 +2316,138 @@
       <c r="N25" s="8"/>
       <c r="O25" s="8"/>
     </row>
+    <row r="26" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+    </row>
+    <row r="27" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+    </row>
+    <row r="28" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="21"/>
+    </row>
+    <row r="29" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="16"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$C2="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A82">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$C2="No"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>$C2="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{FFA2BD12-D726-4B56-B8E9-BC6E0D925A91}">
+      <formula1>"Yes, No, Link Sent"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>